<commit_message>
Update ANTAM gold prices
</commit_message>
<xml_diff>
--- a/data/harga_emas_antam.xlsx
+++ b/data/harga_emas_antam.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harga Emas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Harga Emas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Harga Emas'!$A$1:$D$5033</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Harga Emas'!$A$1:$D$5035</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5033"/>
+  <dimension ref="A1:D5035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64947,8 +64947,36 @@
         <v>147000</v>
       </c>
     </row>
+    <row r="5034">
+      <c r="A5034" s="2" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B5034" s="3" t="n">
+        <v>2624000</v>
+      </c>
+      <c r="C5034" s="3" t="n">
+        <v>2477000</v>
+      </c>
+      <c r="D5034" s="3" t="n">
+        <v>147000</v>
+      </c>
+    </row>
+    <row r="5035">
+      <c r="A5035" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B5035" s="3" t="n">
+        <v>2639000</v>
+      </c>
+      <c r="C5035" s="3" t="n">
+        <v>2492000</v>
+      </c>
+      <c r="D5035" s="3" t="n">
+        <v>147000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D5033"/>
+  <autoFilter ref="A1:D5035"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -64998,7 +65026,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-01 15:20:29 WIB</t>
+          <t>2026-09-03 14:18:09 WIB</t>
         </is>
       </c>
     </row>
@@ -65009,7 +65037,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5032</v>
+        <v>5034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>